<commit_message>
Valoracion del analisis de los PRECIOS terminado
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10303"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Proyectos/cursos_activos/inserta_once/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\analisis-estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54222956-CA8B-9540-87B0-F23EEB278FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF7D7B5-9DFD-49F6-B151-53A74CA64F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="740" windowWidth="38080" windowHeight="19940" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,14 @@
     <sheet name="3_Satisfaccion" sheetId="4" r:id="rId4"/>
     <sheet name="4_Probabilidad" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$4</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'1_Precios'!$B$4</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -628,6 +636,707 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.2</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Histograma</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Histograma</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{CA7B7DDF-73BE-4F4A-9F70-F57FAB979D67}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:v>Precio_Unitario</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Gráfico 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4710B9F8-17BD-28E1-59C1-C80781E2C4EB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4251960" y="2247900"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-ES" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -918,9 +1627,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -964,7 +1673,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -1008,7 +1717,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -1052,7 +1761,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1096,7 +1805,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -1140,7 +1849,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -1184,7 +1893,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -1228,7 +1937,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1272,7 +1981,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1316,7 +2025,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1360,7 +2069,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1404,7 +2113,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1011</v>
       </c>
@@ -1448,7 +2157,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1012</v>
       </c>
@@ -1492,7 +2201,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1013</v>
       </c>
@@ -1536,7 +2245,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1014</v>
       </c>
@@ -1580,7 +2289,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>1015</v>
       </c>
@@ -1624,7 +2333,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1016</v>
       </c>
@@ -1668,7 +2377,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1017</v>
       </c>
@@ -1712,7 +2421,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1018</v>
       </c>
@@ -1756,7 +2465,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1019</v>
       </c>
@@ -1800,7 +2509,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1020</v>
       </c>
@@ -1844,7 +2553,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1021</v>
       </c>
@@ -1888,7 +2597,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1022</v>
       </c>
@@ -1932,7 +2641,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1023</v>
       </c>
@@ -1976,7 +2685,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1024</v>
       </c>
@@ -2020,7 +2729,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1025</v>
       </c>
@@ -2064,7 +2773,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1026</v>
       </c>
@@ -2108,7 +2817,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>1027</v>
       </c>
@@ -2152,7 +2861,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>1028</v>
       </c>
@@ -2196,7 +2905,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1029</v>
       </c>
@@ -2240,7 +2949,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>1030</v>
       </c>
@@ -2284,7 +2993,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>1031</v>
       </c>
@@ -2328,7 +3037,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1032</v>
       </c>
@@ -2372,7 +3081,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1033</v>
       </c>
@@ -2416,7 +3125,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1034</v>
       </c>
@@ -2460,7 +3169,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1035</v>
       </c>
@@ -2504,7 +3213,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1036</v>
       </c>
@@ -2548,7 +3257,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1037</v>
       </c>
@@ -2592,7 +3301,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1038</v>
       </c>
@@ -2636,7 +3345,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1039</v>
       </c>
@@ -2680,7 +3389,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1040</v>
       </c>
@@ -2724,7 +3433,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1041</v>
       </c>
@@ -2768,7 +3477,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1042</v>
       </c>
@@ -2820,7 +3529,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="3" width="15.6640625" customWidth="1"/>
@@ -2828,12 +3537,12 @@
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -2847,7 +3556,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -2857,9 +3566,12 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>60.011904761904759</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -2869,9 +3581,12 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -2881,9 +3596,12 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -2893,9 +3611,12 @@
       <c r="D8" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E8" s="4">
+        <f>_xlfn.STDEV.S(B5:B46)</f>
+        <v>63.23692269082472</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -2903,7 +3624,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -2911,7 +3632,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -2922,7 +3643,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>63</v>
       </c>
@@ -2930,7 +3651,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -2938,7 +3659,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -2946,7 +3667,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -2954,7 +3675,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -2962,7 +3683,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -2970,7 +3691,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -2978,7 +3699,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -2986,7 +3707,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -2994,7 +3715,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -3002,7 +3723,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -3010,7 +3731,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -3018,7 +3739,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -3026,7 +3747,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -3034,7 +3755,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3042,7 +3763,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3050,7 +3771,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -3058,7 +3779,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -3066,7 +3787,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -3074,7 +3795,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -3082,7 +3803,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -3090,7 +3811,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>84</v>
       </c>
@@ -3098,7 +3819,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>85</v>
       </c>
@@ -3106,7 +3827,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>86</v>
       </c>
@@ -3114,7 +3835,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>87</v>
       </c>
@@ -3122,7 +3843,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>88</v>
       </c>
@@ -3130,7 +3851,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>89</v>
       </c>
@@ -3138,7 +3859,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>90</v>
       </c>
@@ -3146,7 +3867,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>91</v>
       </c>
@@ -3154,7 +3875,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -3162,7 +3883,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>93</v>
       </c>
@@ -3170,7 +3891,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>94</v>
       </c>
@@ -3178,7 +3899,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>95</v>
       </c>
@@ -3186,7 +3907,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>95</v>
       </c>
@@ -3194,7 +3915,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>95</v>
       </c>
@@ -3204,13 +3925,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="3" width="15.6640625" customWidth="1"/>
@@ -3218,12 +3940,12 @@
     <col min="6" max="6" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -3240,7 +3962,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -3255,7 +3977,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -3270,7 +3992,7 @@
       </c>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -3285,7 +4007,7 @@
       </c>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -3300,7 +4022,7 @@
       </c>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -3311,7 +4033,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -3322,7 +4044,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -3336,7 +4058,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>63</v>
       </c>
@@ -3347,7 +4069,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -3358,7 +4080,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -3369,7 +4091,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -3380,7 +4102,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -3391,7 +4113,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -3402,7 +4124,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -3413,7 +4135,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -3424,7 +4146,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -3435,7 +4157,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -3446,7 +4168,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -3457,7 +4179,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -3468,7 +4190,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -3479,7 +4201,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -3490,7 +4212,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3501,7 +4223,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3512,7 +4234,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -3523,7 +4245,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -3534,7 +4256,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -3545,7 +4267,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -3556,7 +4278,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -3567,7 +4289,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>84</v>
       </c>
@@ -3578,7 +4300,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>85</v>
       </c>
@@ -3589,7 +4311,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>86</v>
       </c>
@@ -3600,7 +4322,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>87</v>
       </c>
@@ -3611,7 +4333,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>88</v>
       </c>
@@ -3622,7 +4344,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>89</v>
       </c>
@@ -3633,7 +4355,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>90</v>
       </c>
@@ -3644,7 +4366,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>91</v>
       </c>
@@ -3655,7 +4377,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -3666,7 +4388,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>93</v>
       </c>
@@ -3677,7 +4399,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>94</v>
       </c>
@@ -3688,7 +4410,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>95</v>
       </c>
@@ -3699,7 +4421,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>95</v>
       </c>
@@ -3710,7 +4432,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>95</v>
       </c>
@@ -3729,7 +4451,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="3" width="15.6640625" customWidth="1"/>
@@ -3737,12 +4459,12 @@
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -3756,7 +4478,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -3768,7 +4490,7 @@
       </c>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -3780,7 +4502,7 @@
       </c>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -3792,7 +4514,7 @@
       </c>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -3800,7 +4522,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -3808,7 +4530,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -3819,7 +4541,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -3833,7 +4555,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>63</v>
       </c>
@@ -3845,7 +4567,7 @@
       </c>
       <c r="E12" s="4"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -3857,7 +4579,7 @@
       </c>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -3869,7 +4591,7 @@
       </c>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -3881,7 +4603,7 @@
       </c>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -3893,7 +4615,7 @@
       </c>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -3901,7 +4623,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -3909,7 +4631,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -3920,7 +4642,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -3928,7 +4650,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -3936,7 +4658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -3944,7 +4666,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -3952,7 +4674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -3960,7 +4682,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -3968,7 +4690,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3976,7 +4698,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3984,7 +4706,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -3992,7 +4714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -4000,7 +4722,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -4008,7 +4730,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -4016,7 +4738,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -4024,7 +4746,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>84</v>
       </c>
@@ -4032,7 +4754,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>85</v>
       </c>
@@ -4040,7 +4762,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>86</v>
       </c>
@@ -4048,7 +4770,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>87</v>
       </c>
@@ -4056,7 +4778,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>88</v>
       </c>
@@ -4064,7 +4786,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>89</v>
       </c>
@@ -4072,7 +4794,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>90</v>
       </c>
@@ -4080,7 +4802,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>91</v>
       </c>
@@ -4088,7 +4810,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -4096,7 +4818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>93</v>
       </c>
@@ -4104,7 +4826,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>94</v>
       </c>
@@ -4112,7 +4834,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>95</v>
       </c>
@@ -4120,7 +4842,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>95</v>
       </c>
@@ -4128,7 +4850,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>95</v>
       </c>
@@ -4144,25 +4866,25 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98BB36B-BB56-6748-8634-193EA745B178}">
   <dimension ref="A1:G46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="4" width="15.6640625" customWidth="1"/>
     <col min="5" max="7" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D3" s="3" t="s">
         <v>148</v>
       </c>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -4170,7 +4892,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -4190,7 +4912,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -4204,7 +4926,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -4218,7 +4940,7 @@
       <c r="F7" s="8"/>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -4232,7 +4954,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -4246,7 +4968,7 @@
       <c r="F9" s="8"/>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -4254,7 +4976,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -4265,7 +4987,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>63</v>
       </c>
@@ -4276,7 +4998,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -4287,7 +5009,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -4295,7 +5017,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -4306,7 +5028,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -4314,7 +5036,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -4325,7 +5047,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -4333,7 +5055,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -4341,7 +5063,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -4349,7 +5071,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -4357,7 +5079,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -4365,7 +5087,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -4373,7 +5095,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -4381,7 +5103,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -4389,7 +5111,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -4397,7 +5119,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -4405,7 +5127,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -4413,7 +5135,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -4421,7 +5143,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -4429,7 +5151,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -4437,7 +5159,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -4445,7 +5167,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>84</v>
       </c>
@@ -4453,7 +5175,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>85</v>
       </c>
@@ -4461,7 +5183,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>86</v>
       </c>
@@ -4469,7 +5191,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>87</v>
       </c>
@@ -4477,7 +5199,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>88</v>
       </c>
@@ -4485,7 +5207,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>89</v>
       </c>
@@ -4493,7 +5215,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>90</v>
       </c>
@@ -4501,7 +5223,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>91</v>
       </c>
@@ -4509,7 +5231,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -4517,7 +5239,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>93</v>
       </c>
@@ -4525,7 +5247,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>94</v>
       </c>
@@ -4533,7 +5255,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>95</v>
       </c>
@@ -4541,7 +5263,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>95</v>
       </c>
@@ -4549,7 +5271,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
Subimos Grafico y Analisis de Beneficios
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\analisis-estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF7D7B5-9DFD-49F6-B151-53A74CA64F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE133EB5-C536-4966-9E48-E7AC6E694139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,6 @@
     <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$4</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'1_Precios'!$B$4</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -638,6 +635,570 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Dispersión: Coste vs. Beneficio</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'2_Beneficios'!$B$5:$B$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="42"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>80</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'2_Beneficios'!$C$5:$C$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="42"/>
+                <c:pt idx="0">
+                  <c:v>15.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-7BB4-41B8-8C82-94E42BAB9762}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="653967280"/>
+        <c:axId val="653961520"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="653967280"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="653961520"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="653961520"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="653967280"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -709,6 +1270,46 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1256,6 +1857,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1334,6 +2451,47 @@
         </xdr:sp>
       </mc:Fallback>
     </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Gráfico 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52CF7704-0A13-7F2B-9F86-0C980F617D60}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -3975,7 +5133,10 @@
       <c r="E5" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="4">
+        <f>AVERAGE(C5:C46)</f>
+        <v>32.511904761904759</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -3990,7 +5151,10 @@
       <c r="E6" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="4"/>
+      <c r="F6" s="4">
+        <f>_xlfn.STDEV.S(C5:C46)</f>
+        <v>20.550499399082351</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -4005,7 +5169,10 @@
       <c r="E7" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="4">
+        <f>MIN(C5:C46)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -4020,7 +5187,10 @@
       <c r="E8" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="4">
+        <f>MAX(C5:C46)</f>
+        <v>120</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -4445,6 +5615,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Subo valoraciones de Satisfacción
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\analisis-estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE133EB5-C536-4966-9E48-E7AC6E694139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFD7003-BED1-4844-BAF6-82EADCE553E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -498,7 +498,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -542,6 +542,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -606,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -618,6 +626,10 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1199,6 +1211,338 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>📝 Distribución de Satisfacción</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'3_Satisfaccion'!$E$10:$E$11</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>📝 TABLA DE FRECUENCIAS</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Nº de Clientes</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+            <a:scene3d>
+              <a:camera prst="orthographicFront"/>
+              <a:lightRig rig="brightRoom" dir="t">
+                <a:rot lat="0" lon="0" rev="4800000"/>
+              </a:lightRig>
+            </a:scene3d>
+            <a:sp3d prstMaterial="dkEdge">
+              <a:bevelT w="228600"/>
+              <a:bevelB w="0" h="0"/>
+            </a:sp3d>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$D$12:$D$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$E$12:$E$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-99F0-4CE3-85D0-BEAB1150D4E4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1240731776"/>
+        <c:axId val="1240732256"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1240731776"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1240732256"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1240732256"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1240731776"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1349,6 +1693,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -2354,6 +2738,509 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -2477,6 +3364,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52CF7704-0A13-7F2B-9F86-0C980F617D60}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EAB4D59-F7DA-7177-5172-3DDC958CC70B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5621,7 +6549,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
@@ -5659,7 +6587,10 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>4.2857142857142856</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -5671,7 +6602,10 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -5683,7 +6617,10 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -5708,9 +6645,10 @@
       <c r="B10">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="9" t="s">
         <v>134</v>
       </c>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -5736,7 +6674,10 @@
       <c r="D12" s="3">
         <v>1</v>
       </c>
-      <c r="E12" s="4"/>
+      <c r="E12" s="4">
+        <f>COUNTIF($B$5:$B$46,D12)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -5748,7 +6689,10 @@
       <c r="D13" s="3">
         <v>2</v>
       </c>
-      <c r="E13" s="4"/>
+      <c r="E13" s="4">
+        <f t="shared" ref="E13:E16" si="0">COUNTIF($B$5:$B$46,D13)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -5760,7 +6704,10 @@
       <c r="D14" s="3">
         <v>3</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="4">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -5772,7 +6719,10 @@
       <c r="D15" s="3">
         <v>4</v>
       </c>
-      <c r="E15" s="4"/>
+      <c r="E15" s="4">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -5784,9 +6734,12 @@
       <c r="D16" s="3">
         <v>5</v>
       </c>
-      <c r="E16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="4">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -5794,7 +6747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -5802,7 +6755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -5813,7 +6766,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -5821,7 +6774,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -5829,7 +6782,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -5837,7 +6790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -5845,7 +6798,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -5853,7 +6806,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -5861,7 +6814,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -5869,7 +6822,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -5877,7 +6830,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -5885,15 +6838,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
       <c r="B29">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="L29" s="10"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -5901,7 +6855,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -5909,7 +6863,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -6031,6 +6985,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Subo Probabilidad de venta por CANAL
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\analisis-estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFD7003-BED1-4844-BAF6-82EADCE553E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2186679-7C89-4DFA-8D7D-A1BA190A07EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="696" windowWidth="29952" windowHeight="15708" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -1543,6 +1543,769 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:scene3d>
+              <a:camera prst="orthographicFront"/>
+              <a:lightRig rig="threePt" dir="t"/>
+            </a:scene3d>
+            <a:sp3d>
+              <a:bevelT/>
+            </a:sp3d>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d>
+                <a:bevelT/>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-35C8-46EB-9D4B-8E02B8EDF537}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d>
+                <a:bevelT/>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-35C8-46EB-9D4B-8E02B8EDF537}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d>
+                <a:bevelT/>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-35C8-46EB-9D4B-8E02B8EDF537}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:pattFill prst="pct75">
+                <a:fgClr>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="lt1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-ES"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="50000"/>
+                      <a:lumOff val="50000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'4_Probabilidad'!$D$6:$D$8</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>App</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Web</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Tienda</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'4_Probabilidad'!$E$6:$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-35C8-46EB-9D4B-8E02B8EDF537}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="39000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="39000">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="lt1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="25000"/>
+          <a:lumOff val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="50"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="3.3333333333333333E-2"/>
+          <c:y val="0.17171296296296298"/>
+          <c:w val="0.93888888888888888"/>
+          <c:h val="0.6714577865266842"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:sp3d/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:sp3d/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:sp3d/>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:pattFill prst="pct75">
+                <a:fgClr>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="lt1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-ES"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="50000"/>
+                      <a:lumOff val="50000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>('4_Probabilidad'!$D$6,'4_Probabilidad'!$D$7,'4_Probabilidad'!$D$8)</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>App</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Web</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Tienda</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>('4_Probabilidad'!$E$6,'4_Probabilidad'!$E$7,'4_Probabilidad'!$E$8)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FE56-4CA3-8030-D978BEEE2214}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+      </c:pie3DChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="39000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="39000">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="lt1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="25000"/>
+          <a:lumOff val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1733,6 +2496,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -3256,6 +4099,1208 @@
         <a:noFill/>
       </a:ln>
     </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="253">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200" cap="all" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="39000">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="lt1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="pct75">
+        <a:fgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="pct75">
+        <a:fgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="20000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="20000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:lumMod val="95000"/>
+          <a:alpha val="39000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1800" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="264">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200" cap="all" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="39000">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="lt1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="pct75">
+        <a:fgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="pct75">
+        <a:fgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="20000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="20000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:lumMod val="95000"/>
+          <a:alpha val="39000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1800" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -3417,6 +5462,83 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1043940</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>632460</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Gráfico 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C6B2A09-C00C-DC35-DE64-01E24F778FC9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>899160</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>441960</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Gráfico 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F240B74E-6497-16EC-CA88-F0E246D35444}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -7008,7 +9130,10 @@
       <c r="D3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="4">
+        <f>COUNTA(A5:A46)</f>
+        <v>42</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -7048,9 +9173,18 @@
       <c r="D6" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="7"/>
+      <c r="E6" s="4">
+        <f>COUNTIF(B5:B46,D6)</f>
+        <v>11</v>
+      </c>
+      <c r="F6" s="8">
+        <f>E6/$E$9</f>
+        <v>0.26190476190476192</v>
+      </c>
+      <c r="G6" s="7">
+        <f>F6</f>
+        <v>0.26190476190476192</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -7062,9 +9196,18 @@
       <c r="D7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="7"/>
+      <c r="E7" s="4">
+        <f>COUNTIF(B5:B46,D7)</f>
+        <v>17</v>
+      </c>
+      <c r="F7" s="8">
+        <f>E7/$E$9</f>
+        <v>0.40476190476190477</v>
+      </c>
+      <c r="G7" s="7">
+        <f>F7</f>
+        <v>0.40476190476190477</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -7076,9 +9219,18 @@
       <c r="D8" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="7"/>
+      <c r="E8" s="4">
+        <f>COUNTIF(B5:B46,D8)</f>
+        <v>14</v>
+      </c>
+      <c r="F8" s="8">
+        <f>E8/$E$9</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G8" s="7">
+        <f>F8</f>
+        <v>0.33333333333333331</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -7090,9 +9242,18 @@
       <c r="D9" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="7"/>
+      <c r="E9" s="4">
+        <f>SUM(E6:E8)</f>
+        <v>42</v>
+      </c>
+      <c r="F9" s="8">
+        <f>SUM(F6,F7,F8)</f>
+        <v>1</v>
+      </c>
+      <c r="G9" s="7">
+        <f>F9</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -7407,5 +9568,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>